<commit_message>
Wellbeing study: expand validation sample to 8 companies (91 items)
Ran the tightened extractor on salesforce/starbucks/google/stripe/meta/
hubspot (+52 items). 0 comp leaks. Specificity now varies (19 enumerated
items; the earlier all-named result was a 2-company artifact). More
structural cases from meta/hubspot/salesforce.

make_locus_review.py now carries forward existing hand labels on
regeneration (match on company+category+verbatim), so the 39 already-coded
rows survived; 52 new rows are blank and ready to code.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/wellbeing_locus_review.xlsx
+++ b/data/wellbeing_locus_review.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -490,9 +490,17 @@
           <t>Meaningful equity at an early stage company</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -516,9 +524,17 @@
           <t>The option of getting paid in Bitcoin</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -534,16 +550,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>pto_unlimited</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Work whenever you work best (flexible hours)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+          <t>Flexible vacation - take time off when you need it</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -560,16 +584,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>pto_unlimited</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Flexible vacation - take time off when you need it</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+          <t>Work whenever you work best (flexible hours)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -586,16 +618,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>pto_unlimited</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Work whenever you work best (flexible hours)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+          <t>Flexible vacation - take time off when you need it</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -620,8 +660,16 @@
           <t>Flexible vacation - take time off when you need it</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -646,8 +694,16 @@
           <t>Work whenever you work best (flexible hours)</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -664,16 +720,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>pto_unlimited</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Flexible vacation - take time off when you need it</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+          <t>Work whenever you work best (flexible hours)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -690,16 +754,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>pto_unlimited</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Work whenever you work best (flexible hours)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+          <t>Flexible vacation - take time off when you need it</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -724,8 +796,16 @@
           <t>Flexible vacation - take time off when you need it</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -750,8 +830,16 @@
           <t>Work whenever you work best (flexible hours)</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -768,16 +856,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>pto_unlimited</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Flexible vacation - take time off when you need it</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+          <t>Work whenever you work best (flexible hours)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -794,16 +890,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>pto_unlimited</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Work whenever you work best (flexible hours)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+          <t>Flexible vacation - take time off when you need it</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -820,16 +924,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>pto_unlimited</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Flexible vacation - take time off when you need it</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+          <t>Work whenever you work best (flexible hours)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -846,16 +958,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>pto_unlimited</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Work whenever you work best (flexible hours)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+          <t>Flexible vacation - take time off when you need it</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -880,8 +1000,16 @@
           <t>Flexible vacation - take time off when you need it</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -906,8 +1034,16 @@
           <t>Work whenever you work best (flexible hours)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -924,16 +1060,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>pto_unlimited</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Flexible vacation - take time off when you need it</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>Work whenever you work best (flexible hours)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -950,16 +1094,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>caregiver_support</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Work whenever you work best (flexible hours)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+          <t>Fertility: Receive financial support for your fertility needs and access fertility education, evaluations, and more.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -984,8 +1136,16 @@
           <t>Flexible vacation - take time off when you need it</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1002,16 +1162,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>caregiver_support</t>
+          <t>pto_unlimited</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fertility: Receive financial support for your fertility needs and access fertility education, evaluations, and more.</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+          <t>Flexible vacation - take time off when you need it</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1036,8 +1204,16 @@
           <t>Work whenever you work best (flexible hours)</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1054,16 +1230,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>pto_unlimited</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Flexible vacation - take time off when you need it</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>Work whenever you work best (flexible hours)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1088,8 +1272,16 @@
           <t>Most roles are remote-first</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1114,8 +1306,16 @@
           <t>We're a distributed company and you'll mainly work remote.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1140,8 +1340,16 @@
           <t>We're a distributed company and you'll mainly work remote.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1166,8 +1374,16 @@
           <t>You can work from anywhere and are welcome in our San Francisco office.</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1192,8 +1408,16 @@
           <t>We're a distributed company and you'll mainly work remote.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1218,8 +1442,16 @@
           <t>At GitLab B.V. we mostly work from home</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1244,8 +1476,16 @@
           <t>You can work from anywhere and are welcome in our San Francisco office.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1270,8 +1510,16 @@
           <t>Fully distributed: We're a fully remote and completely distributed team, so we can work wherever we're happiest.</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1288,16 +1536,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>wellness_perk</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Buy what you need to be at your best: You don't need to ask permission before spending company money like it's your own - whether it's for a standing desk, a co-working space, or continuing education.</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+          <t>Work asynchronously: Night owls rejoice! We're dedicated to working asynchronously, so we can contribute from anywhere at anytime.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>structural</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1314,16 +1570,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>wellness_perk</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Work asynchronously: Night owls rejoice! We're dedicated to working asynchronously, so we can contribute from anywhere at anytime.</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+          <t>Buy what you need to be at your best: You don't need to ask permission before spending company money like it's your own - whether it's for a standing desk, a co-working space, or continuing education.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1340,16 +1604,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>remote_flexibility</t>
+          <t>other</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Flexibility in schedule to be there for life's important moments</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+          <t>Learn in-demand skills with access to platforms like LinkedIn Learning and GitLab Learn</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1366,16 +1638,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>remote_flexibility</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Learn in-demand skills with access to platforms like LinkedIn Learning and GitLab Learn</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+          <t>Flexibility in schedule to be there for life's important moments</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1400,8 +1680,16 @@
           <t>Flexibility in schedule to be there for life's important moments</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1426,8 +1714,16 @@
           <t>Flexibility in schedule to be there for life's important moments</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1452,8 +1748,16 @@
           <t>Flexibility in schedule to be there for life's important moments</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1478,16 +1782,1376 @@
           <t>Flexibility in schedule to be there for life's important moments</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>individual</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>named_no_number</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Adoption Policy • Google will now assist our employees by offering financial assistance in the adoption of a child. We'll reimburse you up to $5,000</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>mental_health_eap</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Concern Employee Assistance Program: • Confidential counseling &amp; referral service for employees and eligible dependents.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>parental_leave</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Maternity leave: • 12 weeks off at 75% pay</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>parental_leave</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Parental Leave (for non-primary caregivers): • 2 weeks off at 100% pay</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>pto_accrued</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Year: 1st 15 days 4th 20 days 6th 25 days</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Massage &amp; gym:*** • Working hard? Experienced massage therapists on site will melt your stress. • Workout in the gym and enjoy a relaxing sauna all within the Googleplex.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Employees receive free 1 hour passes to enjoy rock climbing or gymnastics at Twisters Gym located in Mountain View</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>parental_leave</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>generous parental leave policies</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>unlimited vacation</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>unlimited vacation</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>pto_minimum_enforced</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Managers at HubSpot encourage all employees to take a minimum of two weeks vacation per year</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>unlimited vacation to all of our employees</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>remote_flexibility</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>work flexible hours that suit them and their families</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>remote_flexibility</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>work remotely when necessary</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>pto_minimum_enforced</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Managers at HubSpot encourage all employees to take a minimum of two weeks vacation per year</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>unlimited vacation to all of our employees</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>remote_flexibility</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>work flexible hours that suit them and their families</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>remote_flexibility</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>work remotely when necessary</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>backup childcare HubSpot provides to its employees, courtesey of care.com</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>remote_flexibility</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>The ability to work from home</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>hubspot</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>remote_flexibility</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>flexible work hours</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>$4,000 baby cash to all new custodial parents</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>up to $3,000 toward day care/babysitting assistance per year</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>mental_health_eap</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Employee Assistance Program</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>parental_leave</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>up to 4 months of Paid Parental Leave</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>pto_accrued</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>21 days of paid vacation</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>unlimited sick days</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>50% reimbursement of most monthly gym fees</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>reimbursed for up to $3,000 toward day care/babysitting assistance per year</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>parental_leave</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>up to 4 months of Paid Parental Leave</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>pto_accrued</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>21 days of paid vacation</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>unlimited sick days</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>50% reimbursement of most monthly gym fees</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Meals on Salesforce.com: takeout meals for new moms and dads</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Foundation Paid time-off for community service work</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>parental_leave</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Paid Maternity/Paternity Programs</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>pto_accrued</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Three (3) weeks off per year (starts accruing on your date of hire)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Health &amp; Fitness Reimbursement programs</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Yoga Classes</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Annual sales club trips to Hawaii</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>pto_accrued</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>6 paid days a year to volunteer</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>pto_accrued</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>3 weeks paid time off in your first year of employment</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>fitness reimbursement</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>salesforce</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>on-site free yoga</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>caregiver_support</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Referral and support resources for child and eldercare</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>more than 50 partner clubs and networks that help our partners share interests and find work/life balance</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>wellness_perk</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>all the handcrafted beverages you can drink</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>other time-off programs</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>sabbatical</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>career sabbaticals</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>full tuition reimbursement</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>starbucks</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>100 percent tuition coverage for all four years of a bachelor's degree</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>stripe</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>pto_unlimited</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Open vacation policy. We don't count days.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid locus" error="Choose: individual, structural, ambiguous, exclude" type="list">
+    <dataValidation sqref="F2:F92" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid locus" error="Choose: individual, structural, ambiguous, exclude" type="list">
       <formula1>"individual,structural,ambiguous,exclude"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid specificity" error="Choose: enumerated_number, named_no_number, generic, exclude" type="list">
+    <dataValidation sqref="G2:G92" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid specificity" error="Choose: enumerated_number, named_no_number, generic, exclude" type="list">
       <formula1>"enumerated_number,named_no_number,generic,exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>